<commit_message>
Se ajustan detalles ya probando el codigo completamente
</commit_message>
<xml_diff>
--- a/data/Accidentes_50.xlsx
+++ b/data/Accidentes_50.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,21 @@
           <t>Clase de Accidente</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Causa probable</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Estado de la vía</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Clima</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -517,6 +532,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,6 +578,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -603,6 +624,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -646,6 +670,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -689,6 +716,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -732,6 +762,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -775,6 +808,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -818,6 +854,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -861,6 +900,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -904,6 +946,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -947,6 +992,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -990,6 +1038,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1033,6 +1084,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1076,6 +1130,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1119,6 +1176,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1162,6 +1222,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1205,6 +1268,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1248,6 +1314,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1291,6 +1360,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1334,6 +1406,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1377,6 +1452,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1420,6 +1498,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1463,6 +1544,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1506,6 +1590,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1549,6 +1636,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1592,6 +1682,9 @@
           <t>ATROPELLO</t>
         </is>
       </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1635,6 +1728,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1678,6 +1774,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1721,6 +1820,9 @@
           <t>ATROPELLO</t>
         </is>
       </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1764,6 +1866,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1807,6 +1912,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1850,6 +1958,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1893,6 +2004,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1936,6 +2050,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1979,6 +2096,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2022,6 +2142,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2065,6 +2188,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2108,6 +2234,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2151,6 +2280,9 @@
           <t>ATROPELLO</t>
         </is>
       </c>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2194,6 +2326,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2237,6 +2372,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2280,6 +2418,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2323,6 +2464,9 @@
           <t>ATROPELLO</t>
         </is>
       </c>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2366,6 +2510,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2409,6 +2556,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2452,6 +2602,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J47" t="inlineStr"/>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2495,6 +2648,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J48" t="inlineStr"/>
+      <c r="K48" t="inlineStr"/>
+      <c r="L48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2538,6 +2694,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J49" t="inlineStr"/>
+      <c r="K49" t="inlineStr"/>
+      <c r="L49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2581,6 +2740,9 @@
           <t>CHOQUE</t>
         </is>
       </c>
+      <c r="J50" t="inlineStr"/>
+      <c r="K50" t="inlineStr"/>
+      <c r="L50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2622,6 +2784,65 @@
       <c r="I51" t="inlineStr">
         <is>
           <t>CHOQUE</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr"/>
+      <c r="K51" t="inlineStr"/>
+      <c r="L51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-11-26 21:06:00</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>A002</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Carrera 71 # 07-09</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>BACHUE</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>HERIDOS</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>ATROPELLO</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Prueba</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Soleado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Se corrigen errores de carga en filtros
</commit_message>
<xml_diff>
--- a/data/Accidentes_50.xlsx
+++ b/data/Accidentes_50.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2846,6 +2846,230 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2025-11-26 21:20:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>A0003</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Calle sur 30</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>SAN CRISTOBAL</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>MUERTOS</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>2</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>CHOQUE</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Prueba</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Mojada</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Lluvioso</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2025-11-26 00:00:00</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>A0004</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>NORTE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>No registra</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>MUERTOS</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>1</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>ATROPELLO</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>PP</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Mojada</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Tormenta</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2025-11-26 22:25:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>A0005</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>OESTE</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN DE AMIGOS</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>MUERTOS</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>1</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>CHOQUE</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>sss</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Mojada</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Tormenta</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2025-11-26 23:13:00</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>A0001</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>ESTE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>CENTRO</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" t="n">
+        <v>2</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>HERIDOS</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>CHOQUE</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>PRR</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Soleado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Se realizan los comentarios de la pagina registrar
</commit_message>
<xml_diff>
--- a/data/Accidentes_50.xlsx
+++ b/data/Accidentes_50.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3070,6 +3070,222 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2025-11-27 17:50:00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>A0006</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN DE AMIGOS</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>HERIDOS</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>ATROPELLO</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Soleado</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2025-11-27 18:07:00</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>A0009</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>OESTE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN DE AMIGOS</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>HERIDOS</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>ATROPELLO</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Soleado</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2025-11-27 18:07:00</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>A0009</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>OESTE</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN DE AMIGOS</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>HERIDOS</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>ATROPELLO</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Soleado</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2025-11-27 18:11:00</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>A0008</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>ESTE</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ASOCIACIÓN DE AMIGOS</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>HERIDOS</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>ATROPELLO</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Soleado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Se realizaron los comentarios de estadisticas
</commit_message>
<xml_diff>
--- a/data/Accidentes_50.xlsx
+++ b/data/Accidentes_50.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3162,11 +3162,7 @@
           <t>ATROPELLO</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr">
         <is>
           <t>Seca</t>
@@ -3218,11 +3214,7 @@
           <t>ATROPELLO</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
+      <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr">
         <is>
           <t>Seca</t>
@@ -3281,6 +3273,62 @@
         </is>
       </c>
       <c r="L60" t="inlineStr">
+        <is>
+          <t>Soleado</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2025-11-28 00:17:00</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>A0010</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Calle 71 # 42-86</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>JUAN MELLAO</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>2</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>MUERTOS</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>1</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>CHOQUE</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Seca</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>Soleado</t>
         </is>

</xml_diff>

<commit_message>
Se ponen emojis a la interfaz
</commit_message>
<xml_diff>
--- a/data/Accidentes_50.xlsx
+++ b/data/Accidentes_50.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3125,17 +3125,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2025-11-27 18:07:00</t>
+          <t>2025-11-27 18:11:00</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>A0009</t>
+          <t>A0008</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>OESTE</t>
+          <t>ESTE</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3144,7 +3144,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F58" t="n">
         <v>1</v>
@@ -3177,41 +3177,41 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2025-11-27 18:07:00</t>
+          <t>2025-11-28 00:17:00</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>A0009</t>
+          <t>A0010</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>OESTE</t>
+          <t>Calle 71 # 42-86</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>ASOCIACIÓN DE AMIGOS</t>
+          <t>JUAN MELLAO</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F59" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>HERIDOS</t>
+          <t>MUERTOS</t>
         </is>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>ATROPELLO</t>
+          <t>CHOQUE</t>
         </is>
       </c>
       <c r="J59" t="inlineStr"/>
@@ -3221,114 +3221,6 @@
         </is>
       </c>
       <c r="L59" t="inlineStr">
-        <is>
-          <t>Soleado</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>2025-11-27 18:11:00</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>A0008</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>ESTE</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>ASOCIACIÓN DE AMIGOS</t>
-        </is>
-      </c>
-      <c r="E60" t="n">
-        <v>2</v>
-      </c>
-      <c r="F60" t="n">
-        <v>1</v>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>HERIDOS</t>
-        </is>
-      </c>
-      <c r="H60" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>ATROPELLO</t>
-        </is>
-      </c>
-      <c r="J60" t="inlineStr"/>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>Seca</t>
-        </is>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Soleado</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>2025-11-28 00:17:00</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>A0010</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Calle 71 # 42-86</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>JUAN MELLAO</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>2</v>
-      </c>
-      <c r="F61" t="n">
-        <v>0</v>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>MUERTOS</t>
-        </is>
-      </c>
-      <c r="H61" t="n">
-        <v>1</v>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>CHOQUE</t>
-        </is>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>Seca</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
         <is>
           <t>Soleado</t>
         </is>

</xml_diff>